<commit_message>
fix(frontend): hoan tat ket noi click the sach Chatbot mo modal chi tiet (BUG-FE-05) va cap nhat bang kiem thu
</commit_message>
<xml_diff>
--- a/docs/BANG_KIEM_THU_VA_FIX_LOI_SMARTLIB.xlsx
+++ b/docs/BANG_KIEM_THU_VA_FIX_LOI_SMARTLIB.xlsx
@@ -644,7 +644,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H44"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -2329,7 +2329,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -3741,7 +3741,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>

</xml_diff>